<commit_message>
test(mapping): migrate invoice samples and verify latest main
</commit_message>
<xml_diff>
--- a/samples/mapping/invoice/page-breaks/template.xlsx
+++ b/samples/mapping/invoice/page-breaks/template.xlsx
@@ -746,9 +746,10 @@
           <t>**@item.price</t>
         </is>
       </c>
-      <c r="F11" s="13">
-        <f>D11*E11</f>
-        <v/>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>**@item.lineTotal</t>
+        </is>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">

</xml_diff>